<commit_message>
Testes de campo, rodada 2 (28 trechos): recall 82%, FP 0%, 13,7 FPS; óculos de maçarico como falta (D28); faixas de distância nas métricas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planilha_testes_campo.xlsx
+++ b/docs/planilha_testes_campo.xlsx
@@ -59583,7 +59583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -59862,189 +59862,170 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>distância 1 m</t>
+          <t>distância até 2 m</t>
         </is>
       </c>
       <c r="B18" s="8">
-        <f>COUNTIFS(Testes!$H$2:$H$500,1,Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$H$2:$H$500,"&lt;=2",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C18" s="19">
-        <f>IFERROR(COUNTIFS(Testes!$H$2:$H$500,1,Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$H$2:$H$500,1,Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$H$2:$H$500,"&lt;=2",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$H$2:$H$500,"&lt;=2",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>COUNTIFS(Testes!$H$2:$H$500,1,Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$H$2:$H$500,"&lt;=2",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>distância 2 m</t>
+          <t>distância de 2 a 4 m</t>
         </is>
       </c>
       <c r="B19" s="20">
-        <f>COUNTIFS(Testes!$H$2:$H$500,2,Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$H$2:$H$500,"&gt;2",Testes!$H$2:$H$500,"&lt;=4",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C19" s="21">
-        <f>IFERROR(COUNTIFS(Testes!$H$2:$H$500,2,Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$H$2:$H$500,2,Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$H$2:$H$500,"&gt;2",Testes!$H$2:$H$500,"&lt;=4",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$H$2:$H$500,"&gt;2",Testes!$H$2:$H$500,"&lt;=4",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D19" s="20">
-        <f>COUNTIFS(Testes!$H$2:$H$500,2,Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$H$2:$H$500,"&gt;2",Testes!$H$2:$H$500,"&lt;=4",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>distância 4 m</t>
+          <t>distância acima de 4 m</t>
         </is>
       </c>
       <c r="B20" s="8">
-        <f>COUNTIFS(Testes!$H$2:$H$500,4,Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$H$2:$H$500,"&gt;4",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C20" s="19">
-        <f>IFERROR(COUNTIFS(Testes!$H$2:$H$500,4,Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$H$2:$H$500,4,Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$H$2:$H$500,"&gt;4",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$H$2:$H$500,"&gt;4",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D20" s="8">
-        <f>COUNTIFS(Testes!$H$2:$H$500,4,Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$H$2:$H$500,"&gt;4",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>distância 6 m</t>
+          <t>ângulo: frente</t>
         </is>
       </c>
       <c r="B21" s="20">
-        <f>COUNTIFS(Testes!$H$2:$H$500,6,Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C21" s="21">
-        <f>IFERROR(COUNTIFS(Testes!$H$2:$H$500,6,Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$H$2:$H$500,6,Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D21" s="20">
-        <f>COUNTIFS(Testes!$H$2:$H$500,6,Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>ângulo: frente</t>
+          <t>ângulo: perfil</t>
         </is>
       </c>
       <c r="B22" s="8">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C22" s="19">
-        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"frente",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>ângulo: perfil</t>
+          <t>ângulo: costas</t>
         </is>
       </c>
       <c r="B23" s="20">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C23" s="21">
-        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D23" s="20">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"perfil",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>ângulo: costas</t>
+          <t>ângulo: varia</t>
         </is>
       </c>
       <c r="B24" s="8">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C24" s="19">
-        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"costas",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>ângulo: varia</t>
+          <t>arco apagado</t>
         </is>
       </c>
       <c r="B25" s="20">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$U$2:$U$500,"&lt;&gt;")</f>
+        <f>COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C25" s="21">
-        <f>IFERROR(COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
+        <f>IFERROR(COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D25" s="20">
-        <f>COUNTIFS(Testes!$G$2:$G$500,"varia",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
+        <f>COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>arco apagado</t>
-        </is>
-      </c>
-      <c r="B26" s="8">
-        <f>COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$U$2:$U$500,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="C26" s="19">
-        <f>IFERROR(COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
-        <v/>
-      </c>
-      <c r="D26" s="8">
-        <f>COUNTIFS(Testes!$I$2:$I$500,"apagado",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
-        <is>
           <t>arco aceso</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B26" s="8">
         <f>COUNTIFS(Testes!$I$2:$I$500,"aceso",Testes!$U$2:$U$500,"&lt;&gt;")</f>
         <v/>
       </c>
-      <c r="C27" s="21">
+      <c r="C26" s="19">
         <f>IFERROR(COUNTIFS(Testes!$I$2:$I$500,"aceso",Testes!$N$2:$N$500,"ocorrência",Testes!$V$2:$V$500,"OK")/COUNTIFS(Testes!$I$2:$I$500,"aceso",Testes!$N$2:$N$500,"ocorrência",Testes!$U$2:$U$500,"&lt;&gt;"),"")</f>
         <v/>
       </c>
-      <c r="D27" s="20">
+      <c r="D26" s="8">
         <f>COUNTIFS(Testes!$I$2:$I$500,"aceso",Testes!$N$2:$N$500,"sem ocorrência",Testes!$V$2:$V$500,"FALHA")</f>
         <v/>
       </c>

</xml_diff>